<commit_message>
Revise concordance benchmark and add stale-index validation
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Dataset_S1.xlsx
+++ b/supplementary/Supplementary_Dataset_S1.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,12 +472,22 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>mapped_diff</t>
+          <t>signed_discrepancy</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>mapped_diff_pct</t>
+          <t>absolute_discrepancy</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>percentage_discrepancy</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>exact_concordance</t>
         </is>
       </c>
     </row>
@@ -516,6 +526,12 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -552,6 +568,12 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -588,6 +610,12 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -624,6 +652,12 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -660,6 +694,12 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -696,6 +736,12 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -732,6 +778,12 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -768,6 +820,12 @@
       <c r="J9" t="n">
         <v>0</v>
       </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -804,6 +862,12 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -840,6 +904,12 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -876,6 +946,12 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -912,6 +988,12 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -948,6 +1030,12 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -984,6 +1072,12 @@
       <c r="J15" t="n">
         <v>0</v>
       </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1020,6 +1114,12 @@
       <c r="J16" t="n">
         <v>0</v>
       </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1056,6 +1156,12 @@
       <c r="J17" t="n">
         <v>0</v>
       </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1092,6 +1198,12 @@
       <c r="J18" t="n">
         <v>0</v>
       </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1128,6 +1240,12 @@
       <c r="J19" t="n">
         <v>0</v>
       </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1164,6 +1282,12 @@
       <c r="J20" t="n">
         <v>0</v>
       </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1200,6 +1324,12 @@
       <c r="J21" t="n">
         <v>0</v>
       </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1236,6 +1366,12 @@
       <c r="J22" t="n">
         <v>0</v>
       </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1272,6 +1408,12 @@
       <c r="J23" t="n">
         <v>0</v>
       </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1308,6 +1450,12 @@
       <c r="J24" t="n">
         <v>0</v>
       </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1344,6 +1492,12 @@
       <c r="J25" t="n">
         <v>0</v>
       </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1380,6 +1534,12 @@
       <c r="J26" t="n">
         <v>0</v>
       </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1416,6 +1576,12 @@
       <c r="J27" t="n">
         <v>0</v>
       </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1451,6 +1617,12 @@
       </c>
       <c r="J28" t="n">
         <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1464,7 +1636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1482,46 +1654,58 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Experiment</t>
+          <t>Study component</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Experiment 2a</t>
+          <t>Baseline concordance experiment</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Manuscript title</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>experiment-2a-reproducibility</t>
+          <t>A Reproducible Computational Benchmarking Framework for Evaluating Concordance Between BAM-Derived Mapped-Read Counts</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Supplementary dataset accompanying the manuscript</t>
+          <t>experiment-2a-reproducibility</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Observation-level mapped-read metrics and discrepancy measures for the 27 paired baseline observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Generated from</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>metrics_table.tsv</t>
         </is>

</xml_diff>